<commit_message>
cost added to the risk table
</commit_message>
<xml_diff>
--- a/public/Data_Cracks and Pothole_1.xlsx
+++ b/public/Data_Cracks and Pothole_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harivardhan.r\OneDrive - Protiviti Member Firm\Desktop\road-survey\Road-Survey\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64BB002E-6307-4178-B43B-DABC5772C1AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3DF0C1E-8499-439A-BDCD-BE7BEFEA73CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B467F67D-8F37-4A99-A002-C9E06355F6C0}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="126">
   <si>
     <t>S.No</t>
   </si>
@@ -397,6 +397,39 @@
   </si>
   <si>
     <t>1122.png</t>
+  </si>
+  <si>
+    <t>County</t>
+  </si>
+  <si>
+    <t>Mendocino County</t>
+  </si>
+  <si>
+    <t>Tehama County</t>
+  </si>
+  <si>
+    <r>
+      <t>Butte County</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Madera County</t>
+  </si>
+  <si>
+    <t>Merced County</t>
+  </si>
+  <si>
+    <t>Stanislaus County</t>
   </si>
 </sst>
 </file>
@@ -406,7 +439,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -433,6 +466,19 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -448,7 +494,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -471,11 +517,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -508,6 +565,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -842,8 +902,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35CE7708-178B-4824-B67D-19590983A603}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -859,9 +918,10 @@
     <col min="11" max="11" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="73.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -901,8 +961,11 @@
       <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" hidden="1">
+      <c r="N1" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -942,8 +1005,11 @@
       <c r="M2" s="9" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" hidden="1">
+      <c r="N2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" s="8">
         <v>3</v>
       </c>
@@ -983,8 +1049,11 @@
       <c r="M3" s="9" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" hidden="1">
+      <c r="N3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" s="8">
         <v>4</v>
       </c>
@@ -1024,8 +1093,11 @@
       <c r="M4" s="9" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" hidden="1">
+      <c r="N4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" s="8">
         <v>5</v>
       </c>
@@ -1065,8 +1137,11 @@
       <c r="M5" s="9" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" hidden="1">
+      <c r="N5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" s="8">
         <v>6</v>
       </c>
@@ -1106,8 +1181,11 @@
       <c r="M6" s="9" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" hidden="1">
+      <c r="N6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" s="8">
         <v>8</v>
       </c>
@@ -1147,8 +1225,11 @@
       <c r="M7" s="9" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" hidden="1">
+      <c r="N7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" s="8">
         <v>9</v>
       </c>
@@ -1188,8 +1269,11 @@
       <c r="M8" s="9" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" hidden="1">
+      <c r="N8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" s="8">
         <v>10</v>
       </c>
@@ -1229,8 +1313,11 @@
       <c r="M9" s="9" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" hidden="1">
+      <c r="N9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" s="8">
         <v>11</v>
       </c>
@@ -1270,8 +1357,11 @@
       <c r="M10" s="9" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" ht="30" hidden="1">
+      <c r="N10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="30">
       <c r="A11" s="8">
         <v>12</v>
       </c>
@@ -1311,8 +1401,11 @@
       <c r="M11" s="9" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" hidden="1">
+      <c r="N11" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" s="8">
         <v>13</v>
       </c>
@@ -1352,8 +1445,11 @@
       <c r="M12" s="9" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" hidden="1">
+      <c r="N12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
       <c r="A13" s="8">
         <v>15</v>
       </c>
@@ -1393,8 +1489,11 @@
       <c r="M13" s="9" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" hidden="1">
+      <c r="N13" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
       <c r="A14" s="8">
         <v>16</v>
       </c>
@@ -1434,8 +1533,11 @@
       <c r="M14" s="9" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" hidden="1">
+      <c r="N14" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
       <c r="A15" s="8">
         <v>17</v>
       </c>
@@ -1475,8 +1577,11 @@
       <c r="M15" s="9" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" hidden="1">
+      <c r="N15" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
       <c r="A16" s="8">
         <v>18</v>
       </c>
@@ -1516,8 +1621,11 @@
       <c r="M16" s="9" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" hidden="1">
+      <c r="N16" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
       <c r="A17" s="8">
         <v>19</v>
       </c>
@@ -1557,8 +1665,11 @@
       <c r="M17" s="9" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" hidden="1">
+      <c r="N17" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
       <c r="A18" s="8">
         <v>20</v>
       </c>
@@ -1598,8 +1709,11 @@
       <c r="M18" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" hidden="1">
+      <c r="N18" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
       <c r="A19" s="8">
         <v>21</v>
       </c>
@@ -1639,8 +1753,11 @@
       <c r="M19" s="9" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" hidden="1">
+      <c r="N19" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
       <c r="A20" s="8">
         <v>22</v>
       </c>
@@ -1680,8 +1797,11 @@
       <c r="M20" s="9" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" hidden="1">
+      <c r="N20" s="16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
       <c r="A21" s="8">
         <v>23</v>
       </c>
@@ -1721,8 +1841,11 @@
       <c r="M21" s="9" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" hidden="1">
+      <c r="N21" s="16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
       <c r="A22" s="8">
         <v>24</v>
       </c>
@@ -1762,8 +1885,11 @@
       <c r="M22" s="9" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" hidden="1">
+      <c r="N22" s="16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
       <c r="A23" s="8">
         <v>25</v>
       </c>
@@ -1803,8 +1929,11 @@
       <c r="M23" s="9" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" hidden="1">
+      <c r="N23" s="16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
       <c r="A24" s="8">
         <v>26</v>
       </c>
@@ -1844,8 +1973,11 @@
       <c r="M24" s="9" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" hidden="1">
+      <c r="N24" s="16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
       <c r="A25" s="8">
         <v>27</v>
       </c>
@@ -1885,8 +2017,11 @@
       <c r="M25" s="9" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" hidden="1">
+      <c r="N25" s="16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
       <c r="A26" s="8">
         <v>29</v>
       </c>
@@ -1926,8 +2061,11 @@
       <c r="M26" s="9" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" hidden="1">
+      <c r="N26" s="16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
       <c r="A27" s="8">
         <v>30</v>
       </c>
@@ -1967,8 +2105,11 @@
       <c r="M27" s="9" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" hidden="1">
+      <c r="N27" s="16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
       <c r="A28" s="8">
         <v>32</v>
       </c>
@@ -2008,8 +2149,11 @@
       <c r="M28" s="9" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="29" spans="1:13" hidden="1">
+      <c r="N28" s="16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
       <c r="A29" s="8">
         <v>33</v>
       </c>
@@ -2049,8 +2193,11 @@
       <c r="M29" s="9" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" hidden="1">
+      <c r="N29" s="16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
       <c r="A30" s="8">
         <v>34</v>
       </c>
@@ -2090,8 +2237,11 @@
       <c r="M30" s="9" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" hidden="1">
+      <c r="N30" s="16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
       <c r="A31" s="8">
         <v>35</v>
       </c>
@@ -2131,8 +2281,11 @@
       <c r="M31" s="9" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="32" spans="1:13" ht="30" hidden="1">
+      <c r="N31" s="16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="30">
       <c r="A32" s="8">
         <v>36</v>
       </c>
@@ -2172,8 +2325,11 @@
       <c r="M32" s="9" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="33" spans="1:13" hidden="1">
+      <c r="N32" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
       <c r="A33" s="8">
         <v>37</v>
       </c>
@@ -2213,8 +2369,11 @@
       <c r="M33" s="13" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" hidden="1">
+      <c r="N33" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
       <c r="A34" s="8">
         <v>38</v>
       </c>
@@ -2254,8 +2413,11 @@
       <c r="M34" s="9" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="35" spans="1:13" hidden="1">
+      <c r="N34" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
       <c r="A35" s="8">
         <v>39</v>
       </c>
@@ -2295,8 +2457,11 @@
       <c r="M35" s="9" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="36" spans="1:13" hidden="1">
+      <c r="N35" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
       <c r="A36" s="8">
         <v>40</v>
       </c>
@@ -2336,8 +2501,11 @@
       <c r="M36" s="9" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" hidden="1">
+      <c r="N36" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
       <c r="A37" s="8">
         <v>41</v>
       </c>
@@ -2377,8 +2545,11 @@
       <c r="M37" s="9" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" hidden="1">
+      <c r="N37" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
       <c r="A38" s="8">
         <v>42</v>
       </c>
@@ -2418,8 +2589,11 @@
       <c r="M38" s="9" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" hidden="1">
+      <c r="N38" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
       <c r="A39" s="8">
         <v>45</v>
       </c>
@@ -2459,8 +2633,11 @@
       <c r="M39" s="9" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" hidden="1">
+      <c r="N39" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
       <c r="A40" s="8">
         <v>46</v>
       </c>
@@ -2500,8 +2677,11 @@
       <c r="M40" s="9" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="41" spans="1:13" hidden="1">
+      <c r="N40" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
       <c r="A41" s="8">
         <v>47</v>
       </c>
@@ -2541,8 +2721,11 @@
       <c r="M41" s="9" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" hidden="1">
+      <c r="N41" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
       <c r="A42" s="8">
         <v>48</v>
       </c>
@@ -2582,8 +2765,11 @@
       <c r="M42" s="9" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="43" spans="1:13" ht="30" hidden="1">
+      <c r="N42" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="30">
       <c r="A43" s="8">
         <v>49</v>
       </c>
@@ -2623,8 +2809,11 @@
       <c r="M43" s="9" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="44" spans="1:13" hidden="1">
+      <c r="N43" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
       <c r="A44" s="8">
         <v>50</v>
       </c>
@@ -2664,8 +2853,11 @@
       <c r="M44" s="9" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="45" spans="1:13">
+      <c r="N44" s="16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14">
       <c r="A45" s="8">
         <v>51</v>
       </c>
@@ -2705,8 +2897,11 @@
       <c r="M45" s="13" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="46" spans="1:13" hidden="1">
+      <c r="N45" s="16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14">
       <c r="A46" s="8">
         <v>53</v>
       </c>
@@ -2744,8 +2939,11 @@
       <c r="M46" s="9" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="47" spans="1:13" hidden="1">
+      <c r="N46" s="16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14">
       <c r="A47" s="8">
         <v>54</v>
       </c>
@@ -2783,8 +2981,11 @@
       <c r="M47" s="9" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="48" spans="1:13" hidden="1">
+      <c r="N47" s="16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14">
       <c r="A48" s="8">
         <v>55</v>
       </c>
@@ -2824,15 +3025,12 @@
       <c r="M48" s="9" t="s">
         <v>109</v>
       </c>
+      <c r="N48" s="16" t="s">
+        <v>124</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N48" xr:uid="{35CE7708-178B-4824-B67D-19590983A603}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="37.53487"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:N48" xr:uid="{35CE7708-178B-4824-B67D-19590983A603}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>